<commit_message>
feature: added search room and common file operations class
</commit_message>
<xml_diff>
--- a/data/rooms.xlsx
+++ b/data/rooms.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,15 +452,11 @@
       <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
       </c>
       <c r="D2" t="n">
         <v>1</v>
@@ -472,6 +468,32 @@
       </c>
       <c r="F2" t="n">
         <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
FIX: handled null case for list rooms
</commit_message>
<xml_diff>
--- a/data/rooms.xlsx
+++ b/data/rooms.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,14 +452,18 @@
       <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C2" t="n">
-        <v>1</v>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>King</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Casual</t>
+        </is>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>1200</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -467,32 +471,6 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
         <v>2</v>
       </c>
     </row>

</xml_diff>